<commit_message>
feat: add Brine Disposal Well to all three system BOMs
Adds Brine Disposal Well ($2.3M, N/A lifespan) to electrical, mechanical,
and hybrid BOMs. Marks it non-COTS and routes it to Brine & Storage stage
in all three systems. Updates accordion description to clarify it is an
entire engineered system (permitted injection well), not a discrete equipment
item.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Downloads\Desalination Project Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CE319F-3F78-4C7C-8DCF-F97A46A95F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D32C5533-DC74-4D19-AA89-DB2A0E81D5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part 1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="57">
   <si>
     <t>Electrical Components</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>kW delta (pump energy) from design [depth=275 m]</t>
+  </si>
+  <si>
+    <t>Brine Disposal Well</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -727,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="59.26953125" customWidth="1"/>
@@ -775,7 +781,7 @@
         <v>1000000</v>
       </c>
       <c r="E2" s="19">
-        <f t="shared" ref="E2:E8" si="0">D2*C2</f>
+        <f t="shared" ref="E2:E9" si="0">D2*C2</f>
         <v>1000000</v>
       </c>
       <c r="F2">
@@ -948,14 +954,14 @@
         <v>17</v>
       </c>
       <c r="C7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="8">
         <v>3500000</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="0"/>
-        <v>7000000</v>
+        <v>3500000</v>
       </c>
       <c r="F7">
         <v>20</v>
@@ -985,244 +991,253 @@
     <row r="8" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="13">
-        <v>1</v>
-      </c>
-      <c r="D8" s="22">
-        <v>2000000</v>
+        <v>55</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8">
+        <v>2300000</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="0"/>
-        <v>2000000</v>
-      </c>
-      <c r="F8">
-        <v>30</v>
-      </c>
-      <c r="L8" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="M8" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="N8" s="4">
-        <v>5000</v>
-      </c>
-      <c r="O8" s="4">
-        <v>500000</v>
-      </c>
-      <c r="P8" s="4">
-        <v>625000</v>
-      </c>
-      <c r="Q8" s="4">
-        <v>75000</v>
-      </c>
-      <c r="R8" s="4">
-        <v>700000</v>
-      </c>
+        <v>2300000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
     </row>
     <row r="9" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
-      <c r="B9" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="15">
-        <f>SUM(E2:E8)</f>
-        <v>13029200</v>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="13">
+        <v>1</v>
+      </c>
+      <c r="D9" s="22">
+        <v>2000000</v>
+      </c>
+      <c r="E9" s="14">
+        <f t="shared" si="0"/>
+        <v>2000000</v>
+      </c>
+      <c r="F9">
+        <v>30</v>
       </c>
       <c r="L9" s="1">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="M9" s="1">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="N9" s="4">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="O9" s="4">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="P9" s="4">
-        <v>750000</v>
+        <v>625000</v>
       </c>
       <c r="Q9" s="4">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="R9" s="4">
-        <v>810000</v>
+        <v>700000</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="15"/>
+      <c r="B10" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="15">
+        <f>SUM(E2:E9)</f>
+        <v>11829200</v>
+      </c>
       <c r="L10" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="M10" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="N10" s="4">
+        <v>6000</v>
+      </c>
+      <c r="O10" s="4">
+        <v>400000</v>
+      </c>
+      <c r="P10" s="4">
+        <v>750000</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>60000</v>
+      </c>
+      <c r="R10" s="4">
+        <v>810000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="15"/>
+      <c r="L11" s="1">
         <v>0.7</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M11" s="1">
         <v>0.3</v>
       </c>
-      <c r="N10" s="4">
+      <c r="N11" s="4">
         <v>7000</v>
       </c>
-      <c r="O10" s="4">
+      <c r="O11" s="4">
         <v>300000</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P11" s="4">
         <v>875000</v>
       </c>
-      <c r="Q10" s="4">
+      <c r="Q11" s="4">
         <v>45000</v>
       </c>
-      <c r="R10" s="4">
+      <c r="R11" s="4">
         <v>920000</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="3"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="L11" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="M11" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="N11" s="4">
-        <v>8000</v>
-      </c>
-      <c r="O11" s="4">
-        <v>200000</v>
-      </c>
-      <c r="P11" s="4">
-        <v>1000000</v>
-      </c>
-      <c r="Q11" s="4">
-        <v>30000</v>
-      </c>
-      <c r="R11" s="4">
-        <v>1030000</v>
-      </c>
-    </row>
     <row r="12" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="1"/>
+      <c r="A12" s="3"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
       <c r="L12" s="1">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="M12" s="1">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="N12" s="4">
-        <v>9000</v>
+        <v>8000</v>
       </c>
       <c r="O12" s="4">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="P12" s="4">
-        <v>1125000</v>
+        <v>1000000</v>
       </c>
       <c r="Q12" s="4">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="R12" s="4">
-        <v>1140000</v>
+        <v>1030000</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
-      <c r="B13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>4</v>
-      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="L13" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="M13" s="1">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="N13" s="4">
-        <v>10000</v>
-      </c>
-      <c r="O13" s="1">
-        <v>0</v>
+        <v>9000</v>
+      </c>
+      <c r="O13" s="4">
+        <v>100000</v>
       </c>
       <c r="P13" s="4">
-        <v>1250000</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>0</v>
+        <v>1125000</v>
+      </c>
+      <c r="Q13" s="4">
+        <v>15000</v>
       </c>
       <c r="R13" s="4">
-        <v>1250000</v>
+        <v>1140000</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="24">
-        <v>1</v>
-      </c>
-      <c r="D14" s="25">
-        <v>1000000</v>
-      </c>
-      <c r="E14" s="10">
-        <v>25</v>
-      </c>
-      <c r="F14" s="10"/>
-      <c r="G14" s="7"/>
+      <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4">
+        <v>10000</v>
+      </c>
+      <c r="O14" s="1">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4">
+        <v>1250000</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>0</v>
+      </c>
+      <c r="R14" s="4">
+        <v>1250000</v>
+      </c>
     </row>
     <row r="15" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="25">
-        <v>15000</v>
+        <v>1000000</v>
       </c>
       <c r="E15" s="10">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="1"/>
+      <c r="G15" s="7"/>
     </row>
     <row r="16" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1</v>
-      </c>
-      <c r="D16" s="22">
-        <v>200000</v>
+      <c r="B16" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="24">
+        <v>3</v>
+      </c>
+      <c r="D16" s="25">
+        <v>15000</v>
       </c>
       <c r="E16" s="10">
         <v>20</v>
@@ -1233,16 +1248,16 @@
     <row r="17" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
       </c>
       <c r="D17" s="22">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="E17" s="10">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="1"/>
@@ -1250,35 +1265,33 @@
     <row r="18" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" s="1">
         <v>1</v>
       </c>
       <c r="D18" s="22">
-        <v>20000</v>
+        <v>300000</v>
       </c>
       <c r="E18" s="10">
-        <v>20</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>27</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F18" s="10"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="22">
-        <v>60000</v>
+        <v>20000</v>
       </c>
       <c r="E19" s="10">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>27</v>
@@ -1288,30 +1301,32 @@
     <row r="20" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="22">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="E20" s="10">
         <v>15</v>
       </c>
-      <c r="F20" s="10"/>
+      <c r="F20" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="1">
         <v>1</v>
       </c>
       <c r="D21" s="22">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="E21" s="10">
         <v>15</v>
@@ -1322,16 +1337,16 @@
     <row r="22" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1">
         <v>1</v>
       </c>
       <c r="D22" s="22">
-        <v>35000</v>
+        <v>60000</v>
       </c>
       <c r="E22" s="10">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="1"/>
@@ -1339,30 +1354,30 @@
     <row r="23" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" s="22">
-        <v>100000</v>
+        <v>35000</v>
       </c>
       <c r="E23" s="10">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
-      <c r="B24" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="24">
-        <v>2</v>
-      </c>
-      <c r="D24" s="25">
-        <v>8000</v>
+      <c r="B24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3</v>
+      </c>
+      <c r="D24" s="22">
+        <v>100000</v>
       </c>
       <c r="E24" s="10">
         <v>15</v>
@@ -1372,17 +1387,17 @@
     </row>
     <row r="25" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
-      <c r="B25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="1">
+      <c r="B25" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="24">
         <v>2</v>
       </c>
-      <c r="D25" s="8">
-        <v>7000000</v>
+      <c r="D25" s="25">
+        <v>8000</v>
       </c>
       <c r="E25" s="10">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F25" s="10"/>
       <c r="G25" s="1"/>
@@ -1390,28 +1405,30 @@
     <row r="26" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C26" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="8">
-        <v>140000</v>
+        <v>3500000</v>
       </c>
       <c r="E26" s="10">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F26" s="10"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
-      <c r="B27" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="25">
-        <v>2000000</v>
+      <c r="B27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="8">
+        <v>140000</v>
       </c>
       <c r="E27" s="10">
         <v>30</v>
@@ -1420,307 +1437,353 @@
       <c r="G27" s="1"/>
     </row>
     <row r="28" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="1"/>
-      <c r="B28" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="26">
-        <f>SUM(D14:D27)</f>
-        <v>10988000</v>
-      </c>
-      <c r="E28" s="10"/>
+      <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1</v>
+      </c>
+      <c r="D28" s="14">
+        <v>2300000</v>
+      </c>
+      <c r="E28" t="s">
+        <v>56</v>
+      </c>
       <c r="F28" s="10"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="3"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="10"/>
+      <c r="A29" s="1"/>
+      <c r="B29" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="24"/>
+      <c r="D29" s="25">
+        <v>2000000</v>
+      </c>
+      <c r="E29" s="10">
+        <v>30</v>
+      </c>
       <c r="F29" s="10"/>
-      <c r="G29" s="3"/>
+      <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="12"/>
+      <c r="B30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" s="26">
+        <f>SUM(D15:D29)</f>
+        <v>9788000</v>
+      </c>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
-      <c r="G30" s="1"/>
+      <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="1"/>
-      <c r="B31" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>4</v>
-      </c>
+      <c r="A31" s="3"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B32" s="24" t="s">
+      <c r="A32" s="1"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B34" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="24">
-        <v>1</v>
-      </c>
-      <c r="D32" s="25">
+      <c r="C34" s="24">
+        <v>1</v>
+      </c>
+      <c r="D34" s="25">
         <v>1000000</v>
       </c>
-      <c r="E32">
+      <c r="E34">
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B33" s="24" t="s">
+    <row r="35" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B35" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="24">
+      <c r="C35" s="24">
         <v>3</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D35" s="25">
         <v>15000</v>
       </c>
-      <c r="E33">
+      <c r="E35">
         <v>20</v>
       </c>
-    </row>
-    <row r="34" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B34" s="1" t="s">
+      <c r="F35" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B36" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="1">
-        <v>1</v>
-      </c>
-      <c r="D34" s="22">
+      <c r="C36" s="1">
+        <v>1</v>
+      </c>
+      <c r="D36" s="22">
         <v>200000</v>
       </c>
-      <c r="E34">
+      <c r="E36">
         <v>20</v>
       </c>
-      <c r="F34" s="10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B35" s="1" t="s">
+    </row>
+    <row r="37" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B37" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="1">
-        <v>1</v>
-      </c>
-      <c r="D35" s="22">
+      <c r="C37" s="1">
+        <v>1</v>
+      </c>
+      <c r="D37" s="22">
         <v>300000</v>
-      </c>
-      <c r="E35">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B36" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="1">
-        <v>1</v>
-      </c>
-      <c r="D36" s="22">
-        <v>50000</v>
-      </c>
-      <c r="E36">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B37" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C37" s="1">
-        <v>1</v>
-      </c>
-      <c r="D37" s="22">
-        <v>60000</v>
       </c>
       <c r="E37">
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B38" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="1">
+        <v>1</v>
+      </c>
+      <c r="D38" s="22">
+        <v>50000</v>
+      </c>
+      <c r="E38">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B39" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" s="1">
+        <v>1</v>
+      </c>
+      <c r="D39" s="22">
+        <v>60000</v>
+      </c>
+      <c r="E39">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B40" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C40" s="1">
         <v>2</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D40" s="8">
         <v>140000</v>
       </c>
-      <c r="E38">
+      <c r="E40">
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B39" s="24" t="s">
+    <row r="41" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B41" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="C39" s="24"/>
-      <c r="D39" s="25">
+      <c r="C41" s="24"/>
+      <c r="D41" s="25">
         <v>2000000</v>
       </c>
-      <c r="E39">
+      <c r="E41">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B40" s="16" t="s">
+    <row r="42" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B42" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C40" s="20">
+      <c r="C42" s="20">
         <v>2</v>
       </c>
-      <c r="D40" s="18">
+      <c r="D42" s="18">
         <v>5200</v>
       </c>
-      <c r="E40">
+      <c r="E42">
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B41" s="1" t="s">
+    <row r="43" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="13">
-        <v>1</v>
-      </c>
-      <c r="D41" s="22">
+      <c r="C43" s="13">
+        <v>1</v>
+      </c>
+      <c r="D43" s="22">
         <v>2600000</v>
-      </c>
-      <c r="E41">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B42" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="1">
-        <v>2</v>
-      </c>
-      <c r="D42" s="8">
-        <v>7000000</v>
-      </c>
-      <c r="E42">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="1">
-        <v>3</v>
-      </c>
-      <c r="D43" s="22">
-        <v>100000</v>
       </c>
       <c r="E43">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="2:6" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B44" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="C44" s="1">
         <v>1</v>
       </c>
-      <c r="D44" s="22">
-        <v>200000</v>
+      <c r="D44" s="8">
+        <v>3500000</v>
       </c>
       <c r="E44">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B45" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C45" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" s="22">
-        <v>60000</v>
+        <v>100000</v>
       </c>
       <c r="E45">
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B46" s="6" t="s">
+    <row r="46" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C46" s="1">
+        <v>1</v>
+      </c>
+      <c r="D46" s="22">
+        <v>200000</v>
+      </c>
+      <c r="E46">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B47" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C47" s="1">
+        <v>1</v>
+      </c>
+      <c r="D47" s="14">
+        <v>2300000</v>
+      </c>
+      <c r="E47" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1</v>
+      </c>
+      <c r="D48" s="22">
+        <v>60000</v>
+      </c>
+      <c r="E48">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B49" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D46" s="15">
-        <f>SUM(D32:D45)</f>
-        <v>13730200</v>
-      </c>
-    </row>
-    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="6" t="s">
+      <c r="D49" s="15">
+        <f>SUM(D34:D48)</f>
+        <v>12530200</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B53" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="27" t="s">
+      <c r="C53" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-    </row>
-    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="27" t="s">
+      <c r="D53" s="27"/>
+      <c r="E53" s="27"/>
+    </row>
+    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B54" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C54" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="27" t="s">
+    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C55" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B53" s="27" t="s">
+    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B56" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C56" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="5" t="s">
+    <row r="57" spans="2:5" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B57" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C57" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="2:5" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B55" t="s">
+    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B58" t="s">
         <v>19</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C58" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>